<commit_message>
Further work on fuel analysis
</commit_message>
<xml_diff>
--- a/data/input_tables/FuelProp.xlsx
+++ b/data/input_tables/FuelProp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{372D8C1C-8BEE-4435-9901-71255279F462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3247A4-E2D0-4D4D-AD0D-A33BAC75400D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="8595" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="62">
   <si>
     <t>Stereotype--&gt;</t>
   </si>
@@ -180,9 +180,6 @@
   </si>
   <si>
     <t>Pump</t>
-  </si>
-  <si>
-    <t>TriFluid</t>
   </si>
   <si>
     <t>Tank</t>
@@ -844,34 +841,34 @@
         <v>46</v>
       </c>
       <c r="AI2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AJ2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AK2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AL2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AM2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AN2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AO2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AP2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AQ2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AR2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.55000000000000004">
@@ -975,37 +972,37 @@
         <v>31</v>
       </c>
       <c r="AH3" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="AI3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ3" t="s">
         <v>49</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="AK3" t="s">
         <v>50</v>
       </c>
-      <c r="AK3" t="s">
+      <c r="AL3" t="s">
         <v>51</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="AM3" t="s">
         <v>52</v>
       </c>
-      <c r="AM3" t="s">
+      <c r="AN3" t="s">
         <v>53</v>
       </c>
-      <c r="AN3" t="s">
-        <v>54</v>
-      </c>
       <c r="AO3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP3" t="s">
         <v>57</v>
       </c>
-      <c r="AP3" t="s">
+      <c r="AQ3" t="s">
         <v>58</v>
       </c>
-      <c r="AQ3" t="s">
+      <c r="AR3" t="s">
         <v>59</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.55000000000000004">
@@ -1112,34 +1109,34 @@
         <v>33</v>
       </c>
       <c r="AI4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AJ4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AK4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AM4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AN4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AO4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AP4" t="s">
         <v>61</v>
       </c>
-      <c r="AP4" t="s">
-        <v>62</v>
-      </c>
       <c r="AQ4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AR4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.55000000000000004">

</xml_diff>

<commit_message>
Fuel System Connection Analysis
</commit_message>
<xml_diff>
--- a/data/input_tables/FuelProp.xlsx
+++ b/data/input_tables/FuelProp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3247A4-E2D0-4D4D-AD0D-A33BAC75400D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7343B52-A08F-4531-9D17-D7DF5FC84883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="8595" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="63">
   <si>
     <t>Stereotype--&gt;</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>(m)</t>
+  </si>
+  <si>
+    <t>TriFluid</t>
   </si>
 </sst>
 </file>
@@ -596,14 +599,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0244E388-F52E-43B9-9DE6-5495768A8D8C}">
-  <dimension ref="A1:AR14"/>
+  <dimension ref="A1:AU14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="29.1015625" customWidth="1"/>
-    <col min="2" max="44" width="20.578125" customWidth="1"/>
+    <col min="2" max="47" width="20.578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -736,8 +739,17 @@
       <c r="AR1" t="s">
         <v>13</v>
       </c>
+      <c r="AS1" t="s">
+        <v>13</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>13</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -859,19 +871,28 @@
         <v>47</v>
       </c>
       <c r="AO2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="AP2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="AQ2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="AR2" t="s">
         <v>55</v>
       </c>
+      <c r="AS2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -972,7 +993,7 @@
         <v>31</v>
       </c>
       <c r="AH3" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="AI3" t="s">
         <v>48</v>
@@ -993,19 +1014,28 @@
         <v>53</v>
       </c>
       <c r="AO3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AR3" t="s">
         <v>56</v>
       </c>
-      <c r="AP3" t="s">
+      <c r="AS3" t="s">
         <v>57</v>
       </c>
-      <c r="AQ3" t="s">
+      <c r="AT3" t="s">
         <v>58</v>
       </c>
-      <c r="AR3" t="s">
+      <c r="AU3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1127,19 +1157,28 @@
         <v>54</v>
       </c>
       <c r="AO4" t="s">
+        <v>33</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>33</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>33</v>
+      </c>
+      <c r="AR4" t="s">
         <v>60</v>
       </c>
-      <c r="AP4" t="s">
+      <c r="AS4" t="s">
         <v>61</v>
       </c>
-      <c r="AQ4" t="s">
+      <c r="AT4" t="s">
         <v>61</v>
       </c>
-      <c r="AR4" t="s">
+      <c r="AU4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1260,20 +1299,29 @@
       <c r="AN5" t="s">
         <v>20</v>
       </c>
-      <c r="AO5">
+      <c r="AO5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR5">
         <v>10</v>
       </c>
-      <c r="AP5">
+      <c r="AS5">
         <v>35</v>
       </c>
-      <c r="AQ5">
+      <c r="AT5">
         <v>25</v>
       </c>
-      <c r="AR5">
+      <c r="AU5">
         <v>-2</v>
       </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1394,20 +1442,29 @@
       <c r="AN6">
         <v>6850</v>
       </c>
-      <c r="AO6">
+      <c r="AO6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>35</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR6">
         <v>200</v>
       </c>
-      <c r="AP6">
+      <c r="AS6">
         <v>45</v>
       </c>
-      <c r="AQ6">
+      <c r="AT6">
         <v>12.5</v>
       </c>
-      <c r="AR6">
+      <c r="AU6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1528,20 +1585,29 @@
       <c r="AN7" t="s">
         <v>20</v>
       </c>
-      <c r="AO7">
+      <c r="AO7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR7">
         <v>6.5</v>
       </c>
-      <c r="AP7">
+      <c r="AS7">
         <v>40</v>
       </c>
-      <c r="AQ7">
+      <c r="AT7">
         <v>1</v>
       </c>
-      <c r="AR7">
+      <c r="AU7">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1662,20 +1728,29 @@
       <c r="AN8" t="s">
         <v>20</v>
       </c>
-      <c r="AO8">
+      <c r="AO8" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR8">
         <v>1.85</v>
       </c>
-      <c r="AP8">
+      <c r="AS8">
         <v>38</v>
       </c>
-      <c r="AQ8">
+      <c r="AT8">
         <v>2</v>
       </c>
-      <c r="AR8">
+      <c r="AU8">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1796,20 +1871,29 @@
       <c r="AN9" t="s">
         <v>20</v>
       </c>
-      <c r="AO9">
+      <c r="AO9" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR9">
         <v>8.1300000000000008</v>
       </c>
-      <c r="AP9">
+      <c r="AS9">
         <v>32.5</v>
       </c>
-      <c r="AQ9">
+      <c r="AT9">
         <v>5</v>
       </c>
-      <c r="AR9">
+      <c r="AU9">
         <v>-3</v>
       </c>
     </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1930,21 +2014,30 @@
       <c r="AN10" t="s">
         <v>20</v>
       </c>
-      <c r="AO10">
+      <c r="AO10" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR10">
         <f>S10*0.23</f>
         <v>1.61</v>
       </c>
-      <c r="AP10">
+      <c r="AS10">
         <v>30</v>
       </c>
-      <c r="AQ10">
+      <c r="AT10">
         <v>4</v>
       </c>
-      <c r="AR10">
+      <c r="AU10">
         <v>0.2</v>
       </c>
     </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2065,21 +2158,30 @@
       <c r="AN11" t="s">
         <v>20</v>
       </c>
-      <c r="AO11">
-        <f t="shared" ref="AO11:AO12" si="0">S11*0.23</f>
+      <c r="AO11" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP11" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ11" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR11">
+        <f t="shared" ref="AR11:AR12" si="0">S11*0.23</f>
         <v>3.68</v>
       </c>
-      <c r="AP11">
+      <c r="AS11">
         <v>30</v>
       </c>
-      <c r="AQ11">
+      <c r="AT11">
         <v>3</v>
       </c>
-      <c r="AR11">
+      <c r="AU11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2200,21 +2302,30 @@
       <c r="AN12" t="s">
         <v>20</v>
       </c>
-      <c r="AO12">
+      <c r="AO12" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP12" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ12" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR12">
         <f t="shared" si="0"/>
         <v>6.9</v>
       </c>
-      <c r="AP12">
+      <c r="AS12">
         <v>30</v>
       </c>
-      <c r="AQ12">
+      <c r="AT12">
         <v>10</v>
       </c>
-      <c r="AR12">
+      <c r="AU12">
         <v>-1.2</v>
       </c>
     </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2335,20 +2446,29 @@
       <c r="AN13" t="s">
         <v>20</v>
       </c>
-      <c r="AO13">
+      <c r="AO13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR13">
         <v>0.6</v>
       </c>
-      <c r="AP13">
+      <c r="AS13">
         <v>26</v>
       </c>
-      <c r="AQ13">
+      <c r="AT13">
         <v>7</v>
       </c>
-      <c r="AR13">
+      <c r="AU13">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2469,16 +2589,25 @@
       <c r="AN14" t="s">
         <v>20</v>
       </c>
-      <c r="AO14">
+      <c r="AO14" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP14" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ14" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR14">
         <v>0.34</v>
       </c>
-      <c r="AP14">
+      <c r="AS14">
         <v>25</v>
       </c>
-      <c r="AQ14">
+      <c r="AT14">
         <v>8</v>
       </c>
-      <c r="AR14">
+      <c r="AU14">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fuel Analysis Complete for now...
</commit_message>
<xml_diff>
--- a/data/input_tables/FuelProp.xlsx
+++ b/data/input_tables/FuelProp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7343B52-A08F-4531-9D17-D7DF5FC84883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A573428-E3FE-4A25-9104-EEC93DFCA08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="8595" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
+    <workbookView xWindow="-57720" yWindow="8880" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="62">
   <si>
     <t>Stereotype--&gt;</t>
   </si>
@@ -225,9 +225,6 @@
   </si>
   <si>
     <t>(m)</t>
-  </si>
-  <si>
-    <t>TriFluid</t>
   </si>
 </sst>
 </file>
@@ -993,7 +990,7 @@
         <v>31</v>
       </c>
       <c r="AH3" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="AI3" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
Begain small test files. Fixed property calculations with Variants
</commit_message>
<xml_diff>
--- a/data/input_tables/FuelProp.xlsx
+++ b/data/input_tables/FuelProp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A573428-E3FE-4A25-9104-EEC93DFCA08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B460E393-5F0E-4A54-A4E2-256481250A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="8880" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -206,9 +206,6 @@
     <t>(kL)</t>
   </si>
   <si>
-    <t>WeightsCenters</t>
-  </si>
-  <si>
     <t>Weight</t>
   </si>
   <si>
@@ -225,6 +222,9 @@
   </si>
   <si>
     <t>(m)</t>
+  </si>
+  <si>
+    <t>Weights</t>
   </si>
 </sst>
 </file>
@@ -877,16 +877,16 @@
         <v>47</v>
       </c>
       <c r="AR2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="AS2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="AT2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="AU2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.55000000000000004">
@@ -1020,16 +1020,16 @@
         <v>32</v>
       </c>
       <c r="AR3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS3" t="s">
         <v>56</v>
       </c>
-      <c r="AS3" t="s">
+      <c r="AT3" t="s">
         <v>57</v>
       </c>
-      <c r="AT3" t="s">
+      <c r="AU3" t="s">
         <v>58</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.55000000000000004">
@@ -1163,16 +1163,16 @@
         <v>33</v>
       </c>
       <c r="AR4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AS4" t="s">
         <v>60</v>
       </c>
-      <c r="AS4" t="s">
-        <v>61</v>
-      </c>
       <c r="AT4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AU4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:47" x14ac:dyDescent="0.55000000000000004">

</xml_diff>

<commit_message>
Added an endurance test
</commit_message>
<xml_diff>
--- a/data/input_tables/FuelProp.xlsx
+++ b/data/input_tables/FuelProp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B460E393-5F0E-4A54-A4E2-256481250A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4340AB-C142-4241-B046-0EFA6FA8A8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
+    <workbookView xWindow="-28920" yWindow="8595" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1422,22 +1422,22 @@
         <v>20</v>
       </c>
       <c r="AI6">
-        <v>20000</v>
+        <v>3500</v>
       </c>
       <c r="AJ6">
-        <v>15000</v>
+        <v>2250</v>
       </c>
       <c r="AK6">
-        <v>7750</v>
+        <v>1575</v>
       </c>
       <c r="AL6">
-        <v>18725</v>
+        <v>2745</v>
       </c>
       <c r="AM6">
-        <v>13475</v>
+        <v>2175</v>
       </c>
       <c r="AN6">
-        <v>6850</v>
+        <v>1130</v>
       </c>
       <c r="AO6" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
ADDED TO THE ADD PROPERTIES
</commit_message>
<xml_diff>
--- a/data/input_tables/FuelProp.xlsx
+++ b/data/input_tables/FuelProp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4340AB-C142-4241-B046-0EFA6FA8A8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDB9BA4-6572-417F-BA07-67B8651A83B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="8595" windowWidth="29040" windowHeight="15720" xr2:uid="{C6A8110E-9783-4C21-A24C-8AD06514364E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="65">
   <si>
     <t>Stereotype--&gt;</t>
   </si>
@@ -65,15 +65,6 @@
     <t>524 (FUEL DISTRIBUTION)</t>
   </si>
   <si>
-    <t>525 (ME FO PIPING)</t>
-  </si>
-  <si>
-    <t>526 (GS FO PIPING)</t>
-  </si>
-  <si>
-    <t>527 (MISSION FO PIPING)</t>
-  </si>
-  <si>
     <t>528 (FO CONTROL)</t>
   </si>
   <si>
@@ -225,6 +216,24 @@
   </si>
   <si>
     <t>Weights</t>
+  </si>
+  <si>
+    <t>525 ABSENT</t>
+  </si>
+  <si>
+    <t>526 ABSENT</t>
+  </si>
+  <si>
+    <t>527 ABSENT</t>
+  </si>
+  <si>
+    <t>525 ME FO PIPING</t>
+  </si>
+  <si>
+    <t>526 GS FO PIPING</t>
+  </si>
+  <si>
+    <t>527 MISSION FO PIPING</t>
   </si>
 </sst>
 </file>
@@ -596,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0244E388-F52E-43B9-9DE6-5495768A8D8C}">
-  <dimension ref="A1:AU14"/>
+  <dimension ref="A1:AU17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="29.1015625" customWidth="1"/>
@@ -605,145 +614,145 @@
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="K1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="P1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="Q1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="R1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="S1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="T1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="U1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="V1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="W1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="X1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="Y1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="Z1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AA1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AB1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AC1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AD1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AE1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AF1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AG1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AH1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AI1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AJ1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AK1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AL1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AM1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AN1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AO1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AP1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AQ1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AR1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AS1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AT1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AU1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.55000000000000004">
@@ -751,142 +760,142 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="N2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="O2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="P2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Q2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="R2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="T2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="U2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="V2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="W2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="X2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="Y2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="Z2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AA2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AB2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AC2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AD2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AE2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AF2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AG2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AH2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AI2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AJ2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AK2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AL2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AM2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AN2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AO2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AP2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AQ2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AR2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="AS2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="AT2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="AU2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.55000000000000004">
@@ -894,142 +903,142 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" t="s">
         <v>24</v>
       </c>
-      <c r="H3" t="s">
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" t="s">
         <v>25</v>
       </c>
-      <c r="I3" t="s">
+      <c r="M3" t="s">
         <v>26</v>
       </c>
-      <c r="J3" t="s">
+      <c r="N3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" t="s">
         <v>27</v>
       </c>
-      <c r="K3" t="s">
+      <c r="P3" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>29</v>
+      </c>
+      <c r="R3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S3" t="s">
+        <v>37</v>
+      </c>
+      <c r="T3" t="s">
+        <v>38</v>
+      </c>
+      <c r="U3" t="s">
+        <v>39</v>
+      </c>
+      <c r="V3" t="s">
+        <v>14</v>
+      </c>
+      <c r="W3" t="s">
+        <v>41</v>
+      </c>
+      <c r="X3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y3" t="s">
         <v>19</v>
       </c>
-      <c r="L3" t="s">
+      <c r="Z3" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>23</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AG3" t="s">
         <v>28</v>
       </c>
-      <c r="M3" t="s">
+      <c r="AH3" t="s">
         <v>29</v>
       </c>
-      <c r="N3" t="s">
-        <v>17</v>
-      </c>
-      <c r="O3" t="s">
-        <v>30</v>
-      </c>
-      <c r="P3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>32</v>
-      </c>
-      <c r="R3" t="s">
-        <v>38</v>
-      </c>
-      <c r="S3" t="s">
-        <v>40</v>
-      </c>
-      <c r="T3" t="s">
-        <v>41</v>
-      </c>
-      <c r="U3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V3" t="s">
-        <v>17</v>
-      </c>
-      <c r="W3" t="s">
-        <v>44</v>
-      </c>
-      <c r="X3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC3" t="s">
+      <c r="AI3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>49</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AO3" t="s">
         <v>27</v>
       </c>
-      <c r="AD3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>17</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>49</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>51</v>
-      </c>
-      <c r="AM3" t="s">
+      <c r="AP3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AR3" t="s">
         <v>52</v>
       </c>
-      <c r="AN3" t="s">
+      <c r="AS3" t="s">
         <v>53</v>
       </c>
-      <c r="AO3" t="s">
-        <v>30</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>32</v>
-      </c>
-      <c r="AR3" t="s">
+      <c r="AT3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AU3" t="s">
         <v>55</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>57</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.55000000000000004">
@@ -1037,142 +1046,142 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="I4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="N4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="O4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="P4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Q4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="R4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="S4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="T4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="U4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="V4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="W4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="X4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="Y4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="Z4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AA4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AB4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AC4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AD4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="AE4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AF4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AG4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AH4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AI4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AJ4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AK4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AL4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AM4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AN4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AO4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AP4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AQ4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AR4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="AS4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="AT4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="AU4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:47" x14ac:dyDescent="0.55000000000000004">
@@ -1180,130 +1189,130 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR5">
         <v>10</v>
@@ -1323,103 +1332,103 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI6">
         <v>3500</v>
@@ -1440,13 +1449,13 @@
         <v>1130</v>
       </c>
       <c r="AO6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="AP6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AQ6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="AR6">
         <v>200</v>
@@ -1466,70 +1475,70 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X7">
         <v>5</v>
@@ -1556,40 +1565,40 @@
         <v>1</v>
       </c>
       <c r="AF7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="AG7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AH7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="AI7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR7">
         <v>6.5</v>
@@ -1609,13 +1618,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E8">
         <v>9</v>
@@ -1648,91 +1657,91 @@
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="P8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="Q8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="R8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR8">
         <v>1.85</v>
@@ -1752,70 +1761,70 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X9">
         <v>13</v>
@@ -1842,40 +1851,40 @@
         <v>1</v>
       </c>
       <c r="AF9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="AG9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AH9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="AI9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR9">
         <v>8.1300000000000008</v>
@@ -1892,55 +1901,55 @@
     </row>
     <row r="10" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R10">
         <v>0.09</v>
@@ -1958,67 +1967,67 @@
         <v>1</v>
       </c>
       <c r="W10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="X10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR10">
         <f>S10*0.23</f>
@@ -2036,575 +2045,1004 @@
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q11" t="s">
-        <v>20</v>
-      </c>
-      <c r="R11">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="S11">
-        <v>16</v>
-      </c>
-      <c r="T11">
-        <v>3</v>
-      </c>
-      <c r="U11">
-        <v>130</v>
-      </c>
-      <c r="V11" t="b">
-        <v>1</v>
+        <v>17</v>
+      </c>
+      <c r="R11" t="s">
+        <v>17</v>
+      </c>
+      <c r="S11" t="s">
+        <v>17</v>
+      </c>
+      <c r="T11" t="s">
+        <v>17</v>
+      </c>
+      <c r="U11" t="s">
+        <v>17</v>
+      </c>
+      <c r="V11" t="s">
+        <v>17</v>
       </c>
       <c r="W11" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="X11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ11" t="s">
-        <v>20</v>
-      </c>
-      <c r="AR11">
-        <f t="shared" ref="AR11:AR12" si="0">S11*0.23</f>
-        <v>3.68</v>
-      </c>
-      <c r="AS11">
-        <v>30</v>
-      </c>
-      <c r="AT11">
-        <v>3</v>
-      </c>
-      <c r="AU11">
-        <v>1</v>
+        <v>17</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS11" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT11" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU11" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R12">
-        <v>0.06</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S12">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="T12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U12">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="V12" t="b">
         <v>1</v>
       </c>
       <c r="W12" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="X12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR12">
-        <f t="shared" si="0"/>
-        <v>6.9</v>
+        <f t="shared" ref="AR12:AR14" si="0">S12*0.23</f>
+        <v>3.68</v>
       </c>
       <c r="AS12">
         <v>30</v>
       </c>
       <c r="AT12">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AU12">
-        <v>-1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>3</v>
+        <v>60</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ13" t="s">
-        <v>20</v>
-      </c>
-      <c r="AR13">
-        <v>0.6</v>
-      </c>
-      <c r="AS13">
-        <v>26</v>
-      </c>
-      <c r="AT13">
-        <v>7</v>
-      </c>
-      <c r="AU13">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU13" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:47" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q14" t="s">
-        <v>20</v>
-      </c>
-      <c r="R14" t="s">
-        <v>20</v>
-      </c>
-      <c r="S14" t="s">
-        <v>20</v>
-      </c>
-      <c r="T14" t="s">
-        <v>20</v>
-      </c>
-      <c r="U14" t="s">
-        <v>20</v>
-      </c>
-      <c r="V14" t="s">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="R14">
+        <v>0.06</v>
+      </c>
+      <c r="S14">
+        <v>30</v>
+      </c>
+      <c r="T14">
+        <v>1</v>
+      </c>
+      <c r="U14">
+        <v>75</v>
+      </c>
+      <c r="V14" t="b">
+        <v>1</v>
       </c>
       <c r="W14" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="X14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Z14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AA14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AE14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AF14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AG14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AI14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AJ14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AK14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AL14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AM14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AN14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AP14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AQ14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AR14">
+        <f t="shared" si="0"/>
+        <v>6.9</v>
+      </c>
+      <c r="AS14">
+        <v>30</v>
+      </c>
+      <c r="AT14">
+        <v>10</v>
+      </c>
+      <c r="AU14">
+        <v>-1.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:47" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" t="s">
+        <v>17</v>
+      </c>
+      <c r="K15" t="s">
+        <v>17</v>
+      </c>
+      <c r="L15" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" t="s">
+        <v>17</v>
+      </c>
+      <c r="N15" t="s">
+        <v>17</v>
+      </c>
+      <c r="O15" t="s">
+        <v>17</v>
+      </c>
+      <c r="P15" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>17</v>
+      </c>
+      <c r="R15" t="s">
+        <v>17</v>
+      </c>
+      <c r="S15" t="s">
+        <v>17</v>
+      </c>
+      <c r="T15" t="s">
+        <v>17</v>
+      </c>
+      <c r="U15" t="s">
+        <v>17</v>
+      </c>
+      <c r="V15" t="s">
+        <v>17</v>
+      </c>
+      <c r="W15" t="s">
+        <v>17</v>
+      </c>
+      <c r="X15" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:47" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L16" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" t="s">
+        <v>17</v>
+      </c>
+      <c r="N16" t="s">
+        <v>17</v>
+      </c>
+      <c r="O16" t="s">
+        <v>17</v>
+      </c>
+      <c r="P16" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>17</v>
+      </c>
+      <c r="R16" t="s">
+        <v>17</v>
+      </c>
+      <c r="S16" t="s">
+        <v>17</v>
+      </c>
+      <c r="T16" t="s">
+        <v>17</v>
+      </c>
+      <c r="U16" t="s">
+        <v>17</v>
+      </c>
+      <c r="V16" t="s">
+        <v>17</v>
+      </c>
+      <c r="W16" t="s">
+        <v>17</v>
+      </c>
+      <c r="X16" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR16">
+        <v>0.6</v>
+      </c>
+      <c r="AS16">
+        <v>26</v>
+      </c>
+      <c r="AT16">
+        <v>7</v>
+      </c>
+      <c r="AU16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:47" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" t="s">
+        <v>17</v>
+      </c>
+      <c r="K17" t="s">
+        <v>17</v>
+      </c>
+      <c r="L17" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" t="s">
+        <v>17</v>
+      </c>
+      <c r="N17" t="s">
+        <v>17</v>
+      </c>
+      <c r="O17" t="s">
+        <v>17</v>
+      </c>
+      <c r="P17" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>17</v>
+      </c>
+      <c r="R17" t="s">
+        <v>17</v>
+      </c>
+      <c r="S17" t="s">
+        <v>17</v>
+      </c>
+      <c r="T17" t="s">
+        <v>17</v>
+      </c>
+      <c r="U17" t="s">
+        <v>17</v>
+      </c>
+      <c r="V17" t="s">
+        <v>17</v>
+      </c>
+      <c r="W17" t="s">
+        <v>17</v>
+      </c>
+      <c r="X17" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR17">
         <v>0.34</v>
       </c>
-      <c r="AS14">
+      <c r="AS17">
         <v>25</v>
       </c>
-      <c r="AT14">
+      <c r="AT17">
         <v>8</v>
       </c>
-      <c r="AU14">
+      <c r="AU17">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>